<commit_message>
feat: add support for dynamic sprint task categories and custom coloring in Gantt chart export
</commit_message>
<xml_diff>
--- a/Backend/templates/gantt_template.xlsx
+++ b/Backend/templates/gantt_template.xlsx
@@ -633,7 +633,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="119">
+  <cellXfs count="115">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -847,7 +847,7 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="13" fillId="8" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="169" fontId="9" fillId="8" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
@@ -870,8 +870,12 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="9" fillId="8" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="13" fillId="8" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="169" fontId="9" fillId="8" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
@@ -903,7 +907,7 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="13" fillId="10" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="169" fontId="9" fillId="10" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
@@ -931,7 +935,7 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="13" fillId="10" borderId="12" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="169" fontId="9" fillId="10" borderId="12" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
@@ -958,32 +962,12 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="11" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="13" fillId="11" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="169" fontId="9" fillId="11" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="171" fontId="13" fillId="11" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="171" fontId="13" fillId="11" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+    <xf numFmtId="164" fontId="9" fillId="11" borderId="12" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="13" fillId="0" borderId="13" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="13" fillId="11" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="8" fillId="4" borderId="14" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
@@ -1003,7 +987,7 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="13" fillId="6" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="169" fontId="9" fillId="6" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
@@ -1027,7 +1011,7 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="9" fillId="6" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="21" fillId="12" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
@@ -1051,7 +1035,7 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="13" fillId="13" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="169" fontId="13" fillId="13" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
@@ -3033,7 +3017,7 @@
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="10"/>
       <c r="B18" s="58"/>
-      <c r="C18" s="58"/>
+      <c r="C18" s="59"/>
       <c r="D18" s="58"/>
       <c r="E18" s="58"/>
       <c r="F18" s="58"/>
@@ -3099,8 +3083,8 @@
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="10"/>
       <c r="B19" s="52"/>
-      <c r="C19" s="59"/>
-      <c r="D19" s="60"/>
+      <c r="C19" s="60"/>
+      <c r="D19" s="61"/>
       <c r="E19" s="57"/>
       <c r="F19" s="57"/>
       <c r="G19" s="57"/>
@@ -3164,14 +3148,14 @@
     </row>
     <row r="20" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="10"/>
-      <c r="B20" s="61" t="s">
+      <c r="B20" s="62" t="s">
         <v>21</v>
       </c>
-      <c r="C20" s="62"/>
-      <c r="D20" s="63"/>
-      <c r="E20" s="64"/>
-      <c r="F20" s="64"/>
-      <c r="G20" s="64"/>
+      <c r="C20" s="63"/>
+      <c r="D20" s="64"/>
+      <c r="E20" s="65"/>
+      <c r="F20" s="65"/>
+      <c r="G20" s="65"/>
       <c r="H20" s="33"/>
       <c r="I20" s="33"/>
       <c r="J20" s="33"/>
@@ -3188,7 +3172,7 @@
       <c r="U20" s="33"/>
       <c r="V20" s="33"/>
       <c r="W20" s="33"/>
-      <c r="X20" s="65"/>
+      <c r="X20" s="66"/>
       <c r="Y20" s="33"/>
       <c r="Z20" s="33"/>
       <c r="AA20" s="33"/>
@@ -3232,16 +3216,16 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="10"/>
-      <c r="B21" s="66" t="s">
+      <c r="B21" s="67" t="s">
         <v>22</v>
       </c>
-      <c r="C21" s="67" t="s">
+      <c r="C21" s="68" t="s">
         <v>20</v>
       </c>
-      <c r="D21" s="68"/>
-      <c r="E21" s="69"/>
-      <c r="F21" s="69"/>
-      <c r="G21" s="70"/>
+      <c r="D21" s="69"/>
+      <c r="E21" s="70"/>
+      <c r="F21" s="70"/>
+      <c r="G21" s="71"/>
       <c r="H21" s="33"/>
       <c r="I21" s="33"/>
       <c r="J21" s="33"/>
@@ -3258,7 +3242,7 @@
       <c r="U21" s="33"/>
       <c r="V21" s="33"/>
       <c r="W21" s="33"/>
-      <c r="X21" s="65"/>
+      <c r="X21" s="66"/>
       <c r="Y21" s="33"/>
       <c r="Z21" s="33"/>
       <c r="AA21" s="33"/>
@@ -3302,16 +3286,16 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="10"/>
-      <c r="B22" s="66" t="s">
+      <c r="B22" s="67" t="s">
         <v>22</v>
       </c>
-      <c r="C22" s="67" t="s">
+      <c r="C22" s="68" t="s">
         <v>20</v>
       </c>
-      <c r="D22" s="68"/>
-      <c r="E22" s="69"/>
-      <c r="F22" s="69"/>
-      <c r="G22" s="70"/>
+      <c r="D22" s="69"/>
+      <c r="E22" s="70"/>
+      <c r="F22" s="70"/>
+      <c r="G22" s="71"/>
       <c r="H22" s="33"/>
       <c r="I22" s="33"/>
       <c r="J22" s="33"/>
@@ -3328,7 +3312,7 @@
       <c r="U22" s="33"/>
       <c r="V22" s="33"/>
       <c r="W22" s="33"/>
-      <c r="X22" s="65"/>
+      <c r="X22" s="66"/>
       <c r="Y22" s="33"/>
       <c r="Z22" s="33"/>
       <c r="AA22" s="33"/>
@@ -3372,16 +3356,16 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="10"/>
-      <c r="B23" s="66" t="s">
+      <c r="B23" s="67" t="s">
         <v>22</v>
       </c>
-      <c r="C23" s="67" t="s">
+      <c r="C23" s="68" t="s">
         <v>20</v>
       </c>
-      <c r="D23" s="68"/>
-      <c r="E23" s="69"/>
-      <c r="F23" s="69"/>
-      <c r="G23" s="70"/>
+      <c r="D23" s="69"/>
+      <c r="E23" s="70"/>
+      <c r="F23" s="70"/>
+      <c r="G23" s="71"/>
       <c r="H23" s="33"/>
       <c r="I23" s="33"/>
       <c r="J23" s="33"/>
@@ -3398,7 +3382,7 @@
       <c r="U23" s="33"/>
       <c r="V23" s="33"/>
       <c r="W23" s="33"/>
-      <c r="X23" s="65"/>
+      <c r="X23" s="66"/>
       <c r="Y23" s="33"/>
       <c r="Z23" s="33"/>
       <c r="AA23" s="33"/>
@@ -3442,16 +3426,16 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="10"/>
-      <c r="B24" s="66" t="s">
+      <c r="B24" s="67" t="s">
         <v>22</v>
       </c>
-      <c r="C24" s="67" t="s">
+      <c r="C24" s="68" t="s">
         <v>20</v>
       </c>
-      <c r="D24" s="68"/>
-      <c r="E24" s="69"/>
-      <c r="F24" s="69"/>
-      <c r="G24" s="70"/>
+      <c r="D24" s="69"/>
+      <c r="E24" s="70"/>
+      <c r="F24" s="70"/>
+      <c r="G24" s="71"/>
       <c r="H24" s="33"/>
       <c r="I24" s="33"/>
       <c r="J24" s="33"/>
@@ -3468,7 +3452,7 @@
       <c r="U24" s="33"/>
       <c r="V24" s="33"/>
       <c r="W24" s="33"/>
-      <c r="X24" s="65"/>
+      <c r="X24" s="66"/>
       <c r="Y24" s="33"/>
       <c r="Z24" s="33"/>
       <c r="AA24" s="33"/>
@@ -3512,16 +3496,16 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="10"/>
-      <c r="B25" s="66" t="s">
+      <c r="B25" s="67" t="s">
         <v>22</v>
       </c>
-      <c r="C25" s="67" t="s">
+      <c r="C25" s="68" t="s">
         <v>20</v>
       </c>
-      <c r="D25" s="68"/>
-      <c r="E25" s="69"/>
-      <c r="F25" s="69"/>
-      <c r="G25" s="70"/>
+      <c r="D25" s="69"/>
+      <c r="E25" s="70"/>
+      <c r="F25" s="70"/>
+      <c r="G25" s="71"/>
       <c r="H25" s="33"/>
       <c r="I25" s="33"/>
       <c r="J25" s="33"/>
@@ -3538,7 +3522,7 @@
       <c r="U25" s="33"/>
       <c r="V25" s="33"/>
       <c r="W25" s="33"/>
-      <c r="X25" s="65"/>
+      <c r="X25" s="66"/>
       <c r="Y25" s="33"/>
       <c r="Z25" s="33"/>
       <c r="AA25" s="33"/>
@@ -3582,16 +3566,16 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="10"/>
-      <c r="B26" s="66" t="s">
+      <c r="B26" s="67" t="s">
         <v>22</v>
       </c>
-      <c r="C26" s="67" t="s">
+      <c r="C26" s="68" t="s">
         <v>20</v>
       </c>
-      <c r="D26" s="68"/>
-      <c r="E26" s="69"/>
-      <c r="F26" s="69"/>
-      <c r="G26" s="70"/>
+      <c r="D26" s="69"/>
+      <c r="E26" s="70"/>
+      <c r="F26" s="70"/>
+      <c r="G26" s="71"/>
       <c r="H26" s="33"/>
       <c r="I26" s="33"/>
       <c r="J26" s="33"/>
@@ -3608,7 +3592,7 @@
       <c r="U26" s="33"/>
       <c r="V26" s="33"/>
       <c r="W26" s="33"/>
-      <c r="X26" s="65"/>
+      <c r="X26" s="66"/>
       <c r="Y26" s="33"/>
       <c r="Z26" s="33"/>
       <c r="AA26" s="33"/>
@@ -3652,16 +3636,16 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="10"/>
-      <c r="B27" s="66" t="s">
+      <c r="B27" s="67" t="s">
         <v>22</v>
       </c>
-      <c r="C27" s="67" t="s">
+      <c r="C27" s="68" t="s">
         <v>20</v>
       </c>
-      <c r="D27" s="68"/>
-      <c r="E27" s="71"/>
-      <c r="F27" s="71"/>
-      <c r="G27" s="72"/>
+      <c r="D27" s="69"/>
+      <c r="E27" s="72"/>
+      <c r="F27" s="72"/>
+      <c r="G27" s="73"/>
       <c r="H27" s="33"/>
       <c r="I27" s="33"/>
       <c r="J27" s="33"/>
@@ -3678,7 +3662,7 @@
       <c r="U27" s="33"/>
       <c r="V27" s="33"/>
       <c r="W27" s="33"/>
-      <c r="X27" s="65"/>
+      <c r="X27" s="66"/>
       <c r="Y27" s="33"/>
       <c r="Z27" s="33"/>
       <c r="AA27" s="33"/>
@@ -3722,12 +3706,12 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="10"/>
-      <c r="B28" s="73"/>
-      <c r="C28" s="74"/>
-      <c r="D28" s="75"/>
-      <c r="E28" s="76"/>
-      <c r="F28" s="76"/>
-      <c r="G28" s="76"/>
+      <c r="B28" s="74"/>
+      <c r="C28" s="75"/>
+      <c r="D28" s="76"/>
+      <c r="E28" s="77"/>
+      <c r="F28" s="77"/>
+      <c r="G28" s="77"/>
       <c r="H28" s="33"/>
       <c r="I28" s="33"/>
       <c r="J28" s="33"/>
@@ -3744,7 +3728,7 @@
       <c r="U28" s="33"/>
       <c r="V28" s="33"/>
       <c r="W28" s="33"/>
-      <c r="X28" s="65"/>
+      <c r="X28" s="66"/>
       <c r="Y28" s="33"/>
       <c r="Z28" s="33"/>
       <c r="AA28" s="33"/>
@@ -3788,12 +3772,12 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="10"/>
-      <c r="B29" s="73"/>
-      <c r="C29" s="74"/>
-      <c r="D29" s="75"/>
-      <c r="E29" s="76"/>
-      <c r="F29" s="76"/>
-      <c r="G29" s="76"/>
+      <c r="B29" s="74"/>
+      <c r="C29" s="75"/>
+      <c r="D29" s="76"/>
+      <c r="E29" s="77"/>
+      <c r="F29" s="77"/>
+      <c r="G29" s="77"/>
       <c r="H29" s="33"/>
       <c r="I29" s="33"/>
       <c r="J29" s="33"/>
@@ -3810,7 +3794,7 @@
       <c r="U29" s="33"/>
       <c r="V29" s="33"/>
       <c r="W29" s="33"/>
-      <c r="X29" s="65"/>
+      <c r="X29" s="66"/>
       <c r="Y29" s="33"/>
       <c r="Z29" s="33"/>
       <c r="AA29" s="33"/>
@@ -3856,14 +3840,14 @@
       <c r="A30" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="B30" s="77" t="s">
+      <c r="B30" s="78" t="s">
         <v>23</v>
       </c>
-      <c r="C30" s="78"/>
-      <c r="D30" s="79"/>
-      <c r="E30" s="80"/>
-      <c r="F30" s="80"/>
-      <c r="G30" s="80"/>
+      <c r="C30" s="79"/>
+      <c r="D30" s="80"/>
+      <c r="E30" s="81"/>
+      <c r="F30" s="81"/>
+      <c r="G30" s="81"/>
       <c r="H30" s="33"/>
       <c r="I30" s="33"/>
       <c r="J30" s="33"/>
@@ -3924,13 +3908,13 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="10"/>
-      <c r="B31" s="81"/>
+      <c r="B31" s="79"/>
       <c r="C31" s="82"/>
-      <c r="D31" s="83"/>
-      <c r="E31" s="84"/>
-      <c r="F31" s="84"/>
-      <c r="G31" s="85"/>
-      <c r="H31" s="86"/>
+      <c r="D31" s="80"/>
+      <c r="E31" s="81"/>
+      <c r="F31" s="81"/>
+      <c r="G31" s="81"/>
+      <c r="H31" s="83"/>
       <c r="I31" s="33"/>
       <c r="J31" s="33"/>
       <c r="K31" s="33"/>
@@ -3990,13 +3974,13 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="10"/>
-      <c r="B32" s="87"/>
+      <c r="B32" s="79"/>
       <c r="C32" s="82"/>
-      <c r="D32" s="83"/>
-      <c r="E32" s="84"/>
-      <c r="F32" s="84"/>
-      <c r="G32" s="85"/>
-      <c r="H32" s="86"/>
+      <c r="D32" s="80"/>
+      <c r="E32" s="81"/>
+      <c r="F32" s="81"/>
+      <c r="G32" s="81"/>
+      <c r="H32" s="83"/>
       <c r="I32" s="33"/>
       <c r="J32" s="33"/>
       <c r="K32" s="33"/>
@@ -4056,13 +4040,13 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="10"/>
-      <c r="B33" s="87"/>
+      <c r="B33" s="79"/>
       <c r="C33" s="82"/>
-      <c r="D33" s="83"/>
-      <c r="E33" s="84"/>
-      <c r="F33" s="84"/>
-      <c r="G33" s="85"/>
-      <c r="H33" s="86"/>
+      <c r="D33" s="80"/>
+      <c r="E33" s="81"/>
+      <c r="F33" s="81"/>
+      <c r="G33" s="81"/>
+      <c r="H33" s="83"/>
       <c r="I33" s="33"/>
       <c r="J33" s="33"/>
       <c r="K33" s="33"/>
@@ -4122,13 +4106,13 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="10"/>
-      <c r="B34" s="87"/>
+      <c r="B34" s="79"/>
       <c r="C34" s="82"/>
-      <c r="D34" s="83"/>
-      <c r="E34" s="84"/>
-      <c r="F34" s="84"/>
-      <c r="G34" s="85"/>
-      <c r="H34" s="86"/>
+      <c r="D34" s="80"/>
+      <c r="E34" s="81"/>
+      <c r="F34" s="81"/>
+      <c r="G34" s="81"/>
+      <c r="H34" s="83"/>
       <c r="I34" s="33"/>
       <c r="J34" s="33"/>
       <c r="K34" s="33"/>
@@ -4190,14 +4174,14 @@
       <c r="A35" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="B35" s="88" t="s">
+      <c r="B35" s="84" t="s">
         <v>24</v>
       </c>
-      <c r="C35" s="89"/>
-      <c r="D35" s="90"/>
-      <c r="E35" s="91"/>
-      <c r="F35" s="91"/>
-      <c r="G35" s="91"/>
+      <c r="C35" s="85"/>
+      <c r="D35" s="86"/>
+      <c r="E35" s="87"/>
+      <c r="F35" s="87"/>
+      <c r="G35" s="87"/>
       <c r="H35" s="33"/>
       <c r="I35" s="33"/>
       <c r="J35" s="33"/>
@@ -4259,11 +4243,11 @@
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="10"/>
       <c r="B36" s="43"/>
-      <c r="C36" s="92"/>
-      <c r="D36" s="93"/>
-      <c r="E36" s="94"/>
-      <c r="F36" s="94"/>
-      <c r="G36" s="95"/>
+      <c r="C36" s="88"/>
+      <c r="D36" s="89"/>
+      <c r="E36" s="90"/>
+      <c r="F36" s="90"/>
+      <c r="G36" s="91"/>
       <c r="H36" s="33"/>
       <c r="I36" s="33"/>
       <c r="J36" s="33"/>
@@ -4276,8 +4260,8 @@
       <c r="Q36" s="33"/>
       <c r="R36" s="33"/>
       <c r="S36" s="33"/>
-      <c r="T36" s="65"/>
-      <c r="U36" s="65"/>
+      <c r="T36" s="66"/>
+      <c r="U36" s="66"/>
       <c r="V36" s="33"/>
       <c r="W36" s="33"/>
       <c r="X36" s="33"/>
@@ -4325,11 +4309,11 @@
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="10"/>
       <c r="B37" s="43"/>
-      <c r="C37" s="92"/>
-      <c r="D37" s="93"/>
-      <c r="E37" s="94"/>
-      <c r="F37" s="94"/>
-      <c r="G37" s="95"/>
+      <c r="C37" s="88"/>
+      <c r="D37" s="89"/>
+      <c r="E37" s="90"/>
+      <c r="F37" s="90"/>
+      <c r="G37" s="91"/>
       <c r="H37" s="33"/>
       <c r="I37" s="33"/>
       <c r="J37" s="33"/>
@@ -4342,8 +4326,8 @@
       <c r="Q37" s="33"/>
       <c r="R37" s="33"/>
       <c r="S37" s="33"/>
-      <c r="T37" s="65"/>
-      <c r="U37" s="65"/>
+      <c r="T37" s="66"/>
+      <c r="U37" s="66"/>
       <c r="V37" s="33"/>
       <c r="W37" s="33"/>
       <c r="X37" s="33"/>
@@ -4391,10 +4375,10 @@
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="10"/>
       <c r="B38" s="43"/>
-      <c r="C38" s="92"/>
-      <c r="D38" s="93"/>
-      <c r="E38" s="94"/>
-      <c r="F38" s="94"/>
+      <c r="C38" s="88"/>
+      <c r="D38" s="89"/>
+      <c r="E38" s="90"/>
+      <c r="F38" s="90"/>
       <c r="G38" s="46"/>
       <c r="H38" s="33"/>
       <c r="I38" s="33"/>
@@ -4408,8 +4392,8 @@
       <c r="Q38" s="33"/>
       <c r="R38" s="33"/>
       <c r="S38" s="33"/>
-      <c r="T38" s="65"/>
-      <c r="U38" s="65"/>
+      <c r="T38" s="66"/>
+      <c r="U38" s="66"/>
       <c r="V38" s="33"/>
       <c r="W38" s="33"/>
       <c r="X38" s="33"/>
@@ -4457,10 +4441,10 @@
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="10"/>
       <c r="B39" s="43"/>
-      <c r="C39" s="92"/>
-      <c r="D39" s="93"/>
-      <c r="E39" s="94"/>
-      <c r="F39" s="94"/>
+      <c r="C39" s="88"/>
+      <c r="D39" s="89"/>
+      <c r="E39" s="90"/>
+      <c r="F39" s="90"/>
       <c r="G39" s="46"/>
       <c r="H39" s="33"/>
       <c r="I39" s="33"/>
@@ -4474,8 +4458,8 @@
       <c r="Q39" s="33"/>
       <c r="R39" s="33"/>
       <c r="S39" s="33"/>
-      <c r="T39" s="65"/>
-      <c r="U39" s="65"/>
+      <c r="T39" s="66"/>
+      <c r="U39" s="66"/>
       <c r="V39" s="33"/>
       <c r="W39" s="33"/>
       <c r="X39" s="33"/>
@@ -4523,10 +4507,10 @@
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="10"/>
       <c r="B40" s="43"/>
-      <c r="C40" s="92"/>
-      <c r="D40" s="93"/>
-      <c r="E40" s="94"/>
-      <c r="F40" s="94"/>
+      <c r="C40" s="88"/>
+      <c r="D40" s="89"/>
+      <c r="E40" s="90"/>
+      <c r="F40" s="90"/>
       <c r="G40" s="46"/>
       <c r="H40" s="33"/>
       <c r="I40" s="33"/>
@@ -4540,8 +4524,8 @@
       <c r="Q40" s="33"/>
       <c r="R40" s="33"/>
       <c r="S40" s="33"/>
-      <c r="T40" s="65"/>
-      <c r="U40" s="65"/>
+      <c r="T40" s="66"/>
+      <c r="U40" s="66"/>
       <c r="V40" s="33"/>
       <c r="W40" s="33"/>
       <c r="X40" s="33"/>
@@ -4589,11 +4573,11 @@
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="10"/>
       <c r="B41" s="43"/>
-      <c r="C41" s="92"/>
-      <c r="D41" s="93"/>
-      <c r="E41" s="94"/>
-      <c r="F41" s="94"/>
-      <c r="G41" s="95"/>
+      <c r="C41" s="88"/>
+      <c r="D41" s="89"/>
+      <c r="E41" s="90"/>
+      <c r="F41" s="90"/>
+      <c r="G41" s="91"/>
       <c r="H41" s="33"/>
       <c r="I41" s="33"/>
       <c r="J41" s="33"/>
@@ -4606,8 +4590,8 @@
       <c r="Q41" s="33"/>
       <c r="R41" s="33"/>
       <c r="S41" s="33"/>
-      <c r="T41" s="65"/>
-      <c r="U41" s="65"/>
+      <c r="T41" s="66"/>
+      <c r="U41" s="66"/>
       <c r="V41" s="33"/>
       <c r="W41" s="33"/>
       <c r="X41" s="33"/>
@@ -4655,11 +4639,11 @@
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="10"/>
       <c r="B42" s="43"/>
-      <c r="C42" s="92"/>
-      <c r="D42" s="93"/>
-      <c r="E42" s="94"/>
-      <c r="F42" s="94"/>
-      <c r="G42" s="95"/>
+      <c r="C42" s="88"/>
+      <c r="D42" s="89"/>
+      <c r="E42" s="90"/>
+      <c r="F42" s="90"/>
+      <c r="G42" s="91"/>
       <c r="H42" s="33"/>
       <c r="I42" s="33"/>
       <c r="J42" s="33"/>
@@ -4672,8 +4656,8 @@
       <c r="Q42" s="33"/>
       <c r="R42" s="33"/>
       <c r="S42" s="33"/>
-      <c r="T42" s="65"/>
-      <c r="U42" s="65"/>
+      <c r="T42" s="66"/>
+      <c r="U42" s="66"/>
       <c r="V42" s="33"/>
       <c r="W42" s="33"/>
       <c r="X42" s="33"/>
@@ -4721,11 +4705,11 @@
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="10"/>
       <c r="B43" s="43"/>
-      <c r="C43" s="92"/>
-      <c r="D43" s="93"/>
-      <c r="E43" s="94"/>
-      <c r="F43" s="94"/>
-      <c r="G43" s="95"/>
+      <c r="C43" s="88"/>
+      <c r="D43" s="89"/>
+      <c r="E43" s="90"/>
+      <c r="F43" s="90"/>
+      <c r="G43" s="91"/>
       <c r="H43" s="33"/>
       <c r="I43" s="33"/>
       <c r="J43" s="33"/>
@@ -4738,8 +4722,8 @@
       <c r="Q43" s="33"/>
       <c r="R43" s="33"/>
       <c r="S43" s="33"/>
-      <c r="T43" s="65"/>
-      <c r="U43" s="65"/>
+      <c r="T43" s="66"/>
+      <c r="U43" s="66"/>
       <c r="V43" s="33"/>
       <c r="W43" s="33"/>
       <c r="X43" s="33"/>
@@ -4787,11 +4771,11 @@
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="10"/>
       <c r="B44" s="43"/>
-      <c r="C44" s="92"/>
-      <c r="D44" s="93"/>
-      <c r="E44" s="94"/>
-      <c r="F44" s="94"/>
-      <c r="G44" s="95"/>
+      <c r="C44" s="88"/>
+      <c r="D44" s="89"/>
+      <c r="E44" s="90"/>
+      <c r="F44" s="90"/>
+      <c r="G44" s="91"/>
       <c r="H44" s="33"/>
       <c r="I44" s="33"/>
       <c r="J44" s="33"/>
@@ -4804,8 +4788,8 @@
       <c r="Q44" s="33"/>
       <c r="R44" s="33"/>
       <c r="S44" s="33"/>
-      <c r="T44" s="65"/>
-      <c r="U44" s="65"/>
+      <c r="T44" s="66"/>
+      <c r="U44" s="66"/>
       <c r="V44" s="33"/>
       <c r="W44" s="33"/>
       <c r="X44" s="33"/>
@@ -4853,11 +4837,11 @@
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="10"/>
       <c r="B45" s="43"/>
-      <c r="C45" s="92"/>
-      <c r="D45" s="93"/>
-      <c r="E45" s="94"/>
-      <c r="F45" s="94"/>
-      <c r="G45" s="95"/>
+      <c r="C45" s="88"/>
+      <c r="D45" s="89"/>
+      <c r="E45" s="90"/>
+      <c r="F45" s="90"/>
+      <c r="G45" s="91"/>
       <c r="H45" s="33"/>
       <c r="I45" s="33"/>
       <c r="J45" s="33"/>
@@ -4870,8 +4854,8 @@
       <c r="Q45" s="33"/>
       <c r="R45" s="33"/>
       <c r="S45" s="33"/>
-      <c r="T45" s="65"/>
-      <c r="U45" s="65"/>
+      <c r="T45" s="66"/>
+      <c r="U45" s="66"/>
       <c r="V45" s="33"/>
       <c r="W45" s="33"/>
       <c r="X45" s="33"/>
@@ -4919,11 +4903,11 @@
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="10"/>
       <c r="B46" s="43"/>
-      <c r="C46" s="92"/>
-      <c r="D46" s="93"/>
-      <c r="E46" s="94"/>
-      <c r="F46" s="94"/>
-      <c r="G46" s="95"/>
+      <c r="C46" s="88"/>
+      <c r="D46" s="89"/>
+      <c r="E46" s="90"/>
+      <c r="F46" s="90"/>
+      <c r="G46" s="91"/>
       <c r="H46" s="33"/>
       <c r="I46" s="33"/>
       <c r="J46" s="33"/>
@@ -4936,8 +4920,8 @@
       <c r="Q46" s="33"/>
       <c r="R46" s="33"/>
       <c r="S46" s="33"/>
-      <c r="T46" s="65"/>
-      <c r="U46" s="65"/>
+      <c r="T46" s="66"/>
+      <c r="U46" s="66"/>
       <c r="V46" s="33"/>
       <c r="W46" s="33"/>
       <c r="X46" s="33"/>
@@ -4985,11 +4969,11 @@
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="10"/>
       <c r="B47" s="43"/>
-      <c r="C47" s="92"/>
-      <c r="D47" s="93"/>
-      <c r="E47" s="94"/>
-      <c r="F47" s="94"/>
-      <c r="G47" s="96"/>
+      <c r="C47" s="88"/>
+      <c r="D47" s="89"/>
+      <c r="E47" s="90"/>
+      <c r="F47" s="90"/>
+      <c r="G47" s="92"/>
       <c r="H47" s="33"/>
       <c r="I47" s="33"/>
       <c r="J47" s="33"/>
@@ -5002,8 +4986,8 @@
       <c r="Q47" s="33"/>
       <c r="R47" s="33"/>
       <c r="S47" s="33"/>
-      <c r="T47" s="65"/>
-      <c r="U47" s="65"/>
+      <c r="T47" s="66"/>
+      <c r="U47" s="66"/>
       <c r="V47" s="33"/>
       <c r="W47" s="33"/>
       <c r="X47" s="33"/>
@@ -5050,12 +5034,12 @@
     </row>
     <row r="48" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A48" s="10"/>
-      <c r="B48" s="97"/>
-      <c r="C48" s="98"/>
+      <c r="B48" s="93"/>
+      <c r="C48" s="94"/>
       <c r="D48" s="45"/>
-      <c r="E48" s="96"/>
-      <c r="F48" s="96"/>
-      <c r="G48" s="96"/>
+      <c r="E48" s="92"/>
+      <c r="F48" s="92"/>
+      <c r="G48" s="92"/>
       <c r="H48" s="33"/>
       <c r="I48" s="33"/>
       <c r="J48" s="33"/>
@@ -5068,8 +5052,8 @@
       <c r="Q48" s="33"/>
       <c r="R48" s="33"/>
       <c r="S48" s="33"/>
-      <c r="T48" s="65"/>
-      <c r="U48" s="65"/>
+      <c r="T48" s="66"/>
+      <c r="U48" s="66"/>
       <c r="V48" s="33"/>
       <c r="W48" s="33"/>
       <c r="X48" s="33"/>
@@ -5116,14 +5100,14 @@
     </row>
     <row r="49" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A49" s="10"/>
-      <c r="B49" s="99" t="s">
+      <c r="B49" s="95" t="s">
         <v>25</v>
       </c>
-      <c r="C49" s="100"/>
-      <c r="D49" s="101"/>
-      <c r="E49" s="102"/>
-      <c r="F49" s="102"/>
-      <c r="G49" s="102"/>
+      <c r="C49" s="96"/>
+      <c r="D49" s="97"/>
+      <c r="E49" s="98"/>
+      <c r="F49" s="98"/>
+      <c r="G49" s="98"/>
       <c r="H49" s="33"/>
       <c r="I49" s="33"/>
       <c r="J49" s="33"/>
@@ -5184,14 +5168,14 @@
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="10"/>
-      <c r="B50" s="103" t="s">
+      <c r="B50" s="99" t="s">
         <v>26</v>
       </c>
-      <c r="C50" s="104"/>
-      <c r="D50" s="105"/>
-      <c r="E50" s="106"/>
-      <c r="F50" s="106"/>
-      <c r="G50" s="106"/>
+      <c r="C50" s="100"/>
+      <c r="D50" s="101"/>
+      <c r="E50" s="102"/>
+      <c r="F50" s="102"/>
+      <c r="G50" s="102"/>
       <c r="H50" s="33"/>
       <c r="I50" s="33"/>
       <c r="J50" s="33"/>
@@ -5252,14 +5236,14 @@
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="10"/>
-      <c r="B51" s="103" t="s">
+      <c r="B51" s="99" t="s">
         <v>27</v>
       </c>
-      <c r="C51" s="104"/>
-      <c r="D51" s="105"/>
-      <c r="E51" s="106"/>
-      <c r="F51" s="106"/>
-      <c r="G51" s="106"/>
+      <c r="C51" s="100"/>
+      <c r="D51" s="101"/>
+      <c r="E51" s="102"/>
+      <c r="F51" s="102"/>
+      <c r="G51" s="102"/>
       <c r="H51" s="33"/>
       <c r="I51" s="33"/>
       <c r="J51" s="33"/>
@@ -5322,71 +5306,71 @@
       <c r="A52" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="B52" s="107" t="s">
+      <c r="B52" s="103" t="s">
         <v>29</v>
       </c>
-      <c r="C52" s="108"/>
-      <c r="D52" s="109"/>
-      <c r="E52" s="110"/>
-      <c r="F52" s="111"/>
-      <c r="G52" s="111"/>
-      <c r="H52" s="112"/>
-      <c r="I52" s="112"/>
-      <c r="J52" s="112"/>
-      <c r="K52" s="112"/>
-      <c r="L52" s="112"/>
-      <c r="M52" s="112"/>
-      <c r="N52" s="112"/>
-      <c r="O52" s="112"/>
-      <c r="P52" s="112"/>
-      <c r="Q52" s="112"/>
-      <c r="R52" s="112"/>
-      <c r="S52" s="112"/>
-      <c r="T52" s="112"/>
-      <c r="U52" s="112"/>
-      <c r="V52" s="112"/>
-      <c r="W52" s="112"/>
-      <c r="X52" s="112"/>
-      <c r="Y52" s="112"/>
-      <c r="Z52" s="112"/>
-      <c r="AA52" s="112"/>
-      <c r="AB52" s="112"/>
-      <c r="AC52" s="112"/>
-      <c r="AD52" s="112"/>
-      <c r="AE52" s="112"/>
-      <c r="AF52" s="112"/>
-      <c r="AG52" s="112"/>
-      <c r="AH52" s="112"/>
-      <c r="AI52" s="112"/>
-      <c r="AJ52" s="112"/>
-      <c r="AK52" s="112"/>
-      <c r="AL52" s="112"/>
-      <c r="AM52" s="112"/>
-      <c r="AN52" s="112"/>
-      <c r="AO52" s="112"/>
-      <c r="AP52" s="112"/>
-      <c r="AQ52" s="112"/>
-      <c r="AR52" s="112"/>
-      <c r="AS52" s="112"/>
-      <c r="AT52" s="112"/>
-      <c r="AU52" s="112"/>
-      <c r="AV52" s="112"/>
-      <c r="AW52" s="112"/>
-      <c r="AX52" s="112"/>
-      <c r="AY52" s="112"/>
-      <c r="AZ52" s="112"/>
-      <c r="BA52" s="112"/>
-      <c r="BB52" s="112"/>
-      <c r="BC52" s="112"/>
-      <c r="BD52" s="112"/>
-      <c r="BE52" s="112"/>
-      <c r="BF52" s="112"/>
-      <c r="BG52" s="112"/>
-      <c r="BH52" s="112"/>
-      <c r="BI52" s="112"/>
-      <c r="BJ52" s="112"/>
-      <c r="BK52" s="112"/>
-      <c r="BL52" s="113"/>
+      <c r="C52" s="104"/>
+      <c r="D52" s="105"/>
+      <c r="E52" s="106"/>
+      <c r="F52" s="107"/>
+      <c r="G52" s="107"/>
+      <c r="H52" s="108"/>
+      <c r="I52" s="108"/>
+      <c r="J52" s="108"/>
+      <c r="K52" s="108"/>
+      <c r="L52" s="108"/>
+      <c r="M52" s="108"/>
+      <c r="N52" s="108"/>
+      <c r="O52" s="108"/>
+      <c r="P52" s="108"/>
+      <c r="Q52" s="108"/>
+      <c r="R52" s="108"/>
+      <c r="S52" s="108"/>
+      <c r="T52" s="108"/>
+      <c r="U52" s="108"/>
+      <c r="V52" s="108"/>
+      <c r="W52" s="108"/>
+      <c r="X52" s="108"/>
+      <c r="Y52" s="108"/>
+      <c r="Z52" s="108"/>
+      <c r="AA52" s="108"/>
+      <c r="AB52" s="108"/>
+      <c r="AC52" s="108"/>
+      <c r="AD52" s="108"/>
+      <c r="AE52" s="108"/>
+      <c r="AF52" s="108"/>
+      <c r="AG52" s="108"/>
+      <c r="AH52" s="108"/>
+      <c r="AI52" s="108"/>
+      <c r="AJ52" s="108"/>
+      <c r="AK52" s="108"/>
+      <c r="AL52" s="108"/>
+      <c r="AM52" s="108"/>
+      <c r="AN52" s="108"/>
+      <c r="AO52" s="108"/>
+      <c r="AP52" s="108"/>
+      <c r="AQ52" s="108"/>
+      <c r="AR52" s="108"/>
+      <c r="AS52" s="108"/>
+      <c r="AT52" s="108"/>
+      <c r="AU52" s="108"/>
+      <c r="AV52" s="108"/>
+      <c r="AW52" s="108"/>
+      <c r="AX52" s="108"/>
+      <c r="AY52" s="108"/>
+      <c r="AZ52" s="108"/>
+      <c r="BA52" s="108"/>
+      <c r="BB52" s="108"/>
+      <c r="BC52" s="108"/>
+      <c r="BD52" s="108"/>
+      <c r="BE52" s="108"/>
+      <c r="BF52" s="108"/>
+      <c r="BG52" s="108"/>
+      <c r="BH52" s="108"/>
+      <c r="BI52" s="108"/>
+      <c r="BJ52" s="108"/>
+      <c r="BK52" s="108"/>
+      <c r="BL52" s="109"/>
     </row>
     <row r="53" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A53" s="10"/>
@@ -5457,11 +5441,11 @@
     <row r="54" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A54" s="10"/>
       <c r="B54" s="8"/>
-      <c r="C54" s="114"/>
+      <c r="C54" s="110"/>
       <c r="D54" s="32"/>
       <c r="E54" s="31"/>
-      <c r="F54" s="115"/>
-      <c r="G54" s="115"/>
+      <c r="F54" s="111"/>
+      <c r="G54" s="111"/>
       <c r="H54" s="8"/>
       <c r="I54" s="8"/>
       <c r="J54" s="8"/>
@@ -5523,7 +5507,7 @@
     <row r="55" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A55" s="10"/>
       <c r="B55" s="8"/>
-      <c r="C55" s="116"/>
+      <c r="C55" s="112"/>
       <c r="D55" s="32"/>
       <c r="E55" s="31"/>
       <c r="F55" s="8"/>
@@ -46774,7 +46758,7 @@
     </row>
     <row r="680" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A680" s="10"/>
-      <c r="B680" s="117" t="n">
+      <c r="B680" s="113" t="n">
         <v>46115</v>
       </c>
       <c r="C680" s="31"/>
@@ -46842,7 +46826,7 @@
     </row>
     <row r="681" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A681" s="10"/>
-      <c r="B681" s="117" t="n">
+      <c r="B681" s="113" t="n">
         <v>46121</v>
       </c>
       <c r="C681" s="31"/>
@@ -46910,7 +46894,7 @@
     </row>
     <row r="682" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A682" s="10"/>
-      <c r="B682" s="117" t="n">
+      <c r="B682" s="113" t="n">
         <v>46127</v>
       </c>
       <c r="C682" s="31"/>
@@ -46978,7 +46962,7 @@
     </row>
     <row r="683" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A683" s="10"/>
-      <c r="B683" s="117" t="n">
+      <c r="B683" s="113" t="n">
         <v>46143</v>
       </c>
       <c r="C683" s="31"/>
@@ -47046,7 +47030,7 @@
     </row>
     <row r="684" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A684" s="10"/>
-      <c r="B684" s="117" t="n">
+      <c r="B684" s="113" t="n">
         <v>45765</v>
       </c>
       <c r="C684" s="31"/>
@@ -47114,7 +47098,7 @@
     </row>
     <row r="685" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A685" s="10"/>
-      <c r="B685" s="117" t="n">
+      <c r="B685" s="113" t="n">
         <v>45778</v>
       </c>
       <c r="C685" s="31"/>
@@ -47182,7 +47166,7 @@
     </row>
     <row r="686" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A686" s="10"/>
-      <c r="B686" s="117" t="n">
+      <c r="B686" s="113" t="n">
         <v>45884</v>
       </c>
       <c r="C686" s="31"/>
@@ -47250,7 +47234,7 @@
     </row>
     <row r="687" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A687" s="10"/>
-      <c r="B687" s="117" t="n">
+      <c r="B687" s="113" t="n">
         <v>45886</v>
       </c>
       <c r="C687" s="31"/>
@@ -47318,7 +47302,7 @@
     </row>
     <row r="688" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A688" s="10"/>
-      <c r="B688" s="117" t="n">
+      <c r="B688" s="113" t="n">
         <v>45905</v>
       </c>
       <c r="C688" s="31"/>
@@ -47386,7 +47370,7 @@
     </row>
     <row r="689" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A689" s="10"/>
-      <c r="B689" s="117" t="n">
+      <c r="B689" s="113" t="n">
         <v>45931</v>
       </c>
       <c r="C689" s="31"/>
@@ -47454,7 +47438,7 @@
     </row>
     <row r="690" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A690" s="10"/>
-      <c r="B690" s="117" t="n">
+      <c r="B690" s="113" t="n">
         <v>45932</v>
       </c>
       <c r="C690" s="31"/>
@@ -47522,7 +47506,7 @@
     </row>
     <row r="691" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A691" s="10"/>
-      <c r="B691" s="118" t="n">
+      <c r="B691" s="114" t="n">
         <v>45951</v>
       </c>
       <c r="C691" s="31"/>
@@ -47590,7 +47574,7 @@
     </row>
     <row r="692" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A692" s="10"/>
-      <c r="B692" s="118" t="n">
+      <c r="B692" s="114" t="n">
         <v>46016</v>
       </c>
       <c r="C692" s="31"/>
@@ -60871,7 +60855,7 @@
     <mergeCell ref="AX3:BD3"/>
     <mergeCell ref="BE3:BK3"/>
   </mergeCells>
-  <conditionalFormatting sqref="H7:BK51 BL31:BL34">
+  <conditionalFormatting sqref="H7:BK13 BL31:BL34 H19:BK51 H14:I18 M14:BK18">
     <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="13">
       <formula>OR(TEXT(H$4,"ddd")="Sat", TEXT(H$4,"ddd")="Sun", COUNTIF($B$680:$B$696,H$4)&gt;0)</formula>
     </cfRule>
@@ -60882,6 +60866,14 @@
   <conditionalFormatting sqref="A1">
     <cfRule type="expression" priority="4" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="15">
       <formula>LEN(TRIM(A1))&gt;0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="J14:L18">
+    <cfRule type="expression" priority="5" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="13">
+      <formula>OR(TEXT(J$4,"ddd")="Sat", TEXT(J$4,"ddd")="Sun", COUNTIF($B$680:$B$696,J$4)&gt;0)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="6" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="14">
+      <formula>AND($F14&gt;=J$4, $E14&lt;K$4)</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">

</xml_diff>